<commit_message>
Pre practitioner usage tracking backup
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/templates/sales_rep_route_template.xlsx
+++ b/public/templates/sales_rep_route_template.xlsx
@@ -5,12 +5,13 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/granville/Desktop/standalone-logbook-app/public/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/granville/Desktop/auto-logbook-sa/public/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC8A9EE-AD39-FA4D-A3B1-49CAC4456B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEA55EF-B51B-634E-A0F3-FAF8BB784EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="WOPQcxg57/VeiW/qaPiV2TMADeeai7dIaaqtArI07hj+EAHjESov0SUskILeyHIANUhltin4N+x1sMdmA3Ryug==" workbookSaltValue="K1q+pkjjwdlqGvPOFQT26Q==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-34060" yWindow="9100" windowWidth="28040" windowHeight="17360" xr2:uid="{54FC0AFF-17BF-C246-8BB3-3EE54009E567}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="29400" windowHeight="18480" xr2:uid="{54FC0AFF-17BF-C246-8BB3-3EE54009E567}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
   <si>
     <t>Customer</t>
   </si>
@@ -69,36 +70,6 @@
   </si>
   <si>
     <t>BELMONT BLUE BOTTLE LIQUORS (PTY) LTD</t>
-  </si>
-  <si>
-    <t>KORA TRADING BK t/a KORA DW *KBA*</t>
-  </si>
-  <si>
-    <t>MIDON DRANKWINKEL *KBA*</t>
-  </si>
-  <si>
-    <t>ONE STOP LUTZVILLE</t>
-  </si>
-  <si>
-    <t>WEST COAST HOTEL BK *KBA*</t>
-  </si>
-  <si>
-    <t>WINKELSHOEK WYNKELDER EDMS BPK</t>
-  </si>
-  <si>
-    <t>BELMONT ROADWAY BLUE BOTTLE LIQ*KBA*</t>
-  </si>
-  <si>
-    <t>HUIWEITRADING(PTY)LTD VREDENBURG LIQ*COD</t>
-  </si>
-  <si>
-    <t>MATZIK LIQUOR BK h/a BLUE BOTTLE*KBA*</t>
-  </si>
-  <si>
-    <t>BLUE BOTTLE LAMBERTSBAAI *7DAYS*</t>
-  </si>
-  <si>
-    <t>NIEUWOUDTVILLE MANSWINKEL(PTY)LTD*KBA*</t>
   </si>
   <si>
     <t>1,2</t>
@@ -154,7 +125,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="-0.499984740745262"/>
+        <fgColor theme="7" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -332,6 +303,41 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="13">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -725,41 +731,6 @@
         </bottom>
       </border>
     </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -796,7 +767,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EE816E7F-9738-744B-AB22-7F8A329811CB}" name="Table1" displayName="Table1" ref="A1:H278" totalsRowShown="0" headerRowDxfId="12" dataDxfId="10" headerRowBorderDxfId="11" tableBorderDxfId="9" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EE816E7F-9738-744B-AB22-7F8A329811CB}" name="Table1" displayName="Table1" ref="A1:H278" totalsRowShown="0" headerRowDxfId="0" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="A1:H278" xr:uid="{EE816E7F-9738-744B-AB22-7F8A329811CB}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -808,14 +779,14 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{DC165014-20D2-CC46-8068-959CE3B2D92A}" name="Customer" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{98E58A5F-5DF4-DC4E-8F05-9AF75969A6B6}" name="Monday" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{9B49EE92-AEBA-F349-B577-6FBD76DC51A7}" name="Tuesday" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{C8A60DD2-F864-6647-8873-B1D8F55EB421}" name="Wednesday" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{880CCA63-FBE4-784B-8A2D-6ED0B1CDF8C5}" name="Thursday" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{00885726-6084-8B45-A9C2-6A70698A3C44}" name="Friday" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{96A8A272-F29F-D747-AF0B-C9D657C4570B}" name="Saturday" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{DD8E6DDB-7303-2F45-841F-4CE6E4D60B5C}" name="Week" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{DC165014-20D2-CC46-8068-959CE3B2D92A}" name="Customer" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{98E58A5F-5DF4-DC4E-8F05-9AF75969A6B6}" name="Monday" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{9B49EE92-AEBA-F349-B577-6FBD76DC51A7}" name="Tuesday" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{C8A60DD2-F864-6647-8873-B1D8F55EB421}" name="Wednesday" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{880CCA63-FBE4-784B-8A2D-6ED0B1CDF8C5}" name="Thursday" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00885726-6084-8B45-A9C2-6A70698A3C44}" name="Friday" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{96A8A272-F29F-D747-AF0B-C9D657C4570B}" name="Saturday" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{DD8E6DDB-7303-2F45-841F-4CE6E4D60B5C}" name="Week" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight19" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1192,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" s="4" t="b">
         <v>0</v>
@@ -1205,11 +1176,9 @@
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="A3" s="3"/>
       <c r="B3" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="4" t="b">
         <v>0</v>
@@ -1226,77 +1195,65 @@
       <c r="G3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>21</v>
-      </c>
+      <c r="H3" s="5"/>
       <c r="Z3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="Z4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="Z5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="C4" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D4" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="5">
-        <v>2</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>22</v>
-      </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>14</v>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="4" t="b">
         <v>0</v>
@@ -1313,22 +1270,18 @@
       <c r="G6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="H6" s="5"/>
       <c r="Z6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>15</v>
-      </c>
+      <c r="A7" s="3"/>
       <c r="B7" s="4" t="b">
         <v>0</v>
       </c>
       <c r="C7" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="4" t="b">
         <v>0</v>
@@ -1342,19 +1295,15 @@
       <c r="G7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="5">
-        <v>4</v>
-      </c>
+      <c r="H7" s="5"/>
       <c r="Z7" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A8" s="3"/>
       <c r="B8" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" s="4" t="b">
         <v>0</v>
@@ -1371,17 +1320,13 @@
       <c r="G8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="5">
-        <v>3</v>
-      </c>
+      <c r="H8" s="5"/>
       <c r="Z8" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A9" s="3"/>
       <c r="B9" s="4" t="b">
         <v>0</v>
       </c>
@@ -1389,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="b">
         <v>0</v>
@@ -1400,22 +1345,18 @@
       <c r="G9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="5">
-        <v>3</v>
-      </c>
+      <c r="H9" s="5"/>
       <c r="Z9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="A10" s="3"/>
       <c r="B10" s="4" t="b">
         <v>0</v>
       </c>
       <c r="C10" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4" t="b">
         <v>0</v>
@@ -1429,19 +1370,15 @@
       <c r="G10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="5">
-        <v>2</v>
-      </c>
+      <c r="H10" s="5"/>
       <c r="Z10" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="A11" s="3"/>
       <c r="B11" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="4" t="b">
         <v>0</v>
@@ -1458,17 +1395,13 @@
       <c r="G11" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="5">
-        <v>2</v>
-      </c>
+      <c r="H11" s="5"/>
       <c r="Z11">
         <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A12" s="3"/>
       <c r="B12" s="4" t="b">
         <v>0</v>
       </c>
@@ -1476,7 +1409,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4" t="b">
         <v>0</v>
@@ -1487,9 +1420,7 @@
       <c r="G12" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="5">
-        <v>1</v>
-      </c>
+      <c r="H12" s="5"/>
       <c r="Z12">
         <v>3</v>
       </c>
@@ -1516,7 +1447,7 @@
       </c>
       <c r="H13" s="5"/>
       <c r="Z13" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
@@ -7573,14 +7504,14 @@
       <c r="H300" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="UiuzTz7sPATe5iINSGrhya8dWUY5/LigKEtHK3B8eA+E9I2BQMkvxEnqhWuV/Uq0LkENVNuaAuLK7gqE4g5ogQ==" saltValue="KN0F4Hq93RzQ4OZnGhgDwg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="A2:A3 A5:A11 A13:A113" name="Range1_1"/>
   </protectedRanges>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H300" xr:uid="{3B05D1E8-7A16-ED42-9B4F-3DD70FEE9E6B}">
       <formula1>$Z$3:$Z$14</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Visit Frequency Guide" prompt="Weekly → Use Week 1,2,3,4  _x000a_Bi-Weekly → Use Week 1 &amp; 3 (or 2 &amp; 4)  _x000a_Monthly → Use Week 1 only" sqref="H1" xr:uid="{CB6E72FC-2CD5-CF47-96A7-75ACD4F83CDF}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>